<commit_message>
Added some comments to Notebook 4
</commit_message>
<xml_diff>
--- a/Gian/suggestions.xlsx
+++ b/Gian/suggestions.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\noahm\projects\loc_analysis\Gian\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{6CF9FF98-546E-456A-9145-F56FEC502ECE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{73F12D7B-66B3-486A-82D7-7BCDF3CBBD0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{6B063EC0-67D1-47C9-8561-C8AF2753B48C}"/>
+    <workbookView xWindow="-28920" yWindow="-15" windowWidth="29040" windowHeight="15720" xr2:uid="{6B063EC0-67D1-47C9-8561-C8AF2753B48C}"/>
   </bookViews>
   <sheets>
-    <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
+    <sheet name="Overview" sheetId="1" r:id="rId1"/>
+    <sheet name="Status Update" sheetId="3" r:id="rId2"/>
+    <sheet name="Tabelle2" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="39">
   <si>
     <t>Notebook</t>
   </si>
@@ -143,13 +145,28 @@
   </si>
   <si>
     <t>Be cautious with ICLabel: quite substantial number of artefacts are excluded.</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Resolved</t>
+  </si>
+  <si>
+    <t>Pending</t>
+  </si>
+  <si>
+    <t>Send Gian follow-up mail</t>
+  </si>
+  <si>
+    <t>To-Do</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -164,6 +181,19 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Neue Haas Grotesk Text Pro"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Neue Haas Grotesk Text Pro"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -180,20 +210,11 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="20">
+  <borders count="13">
     <border>
       <left/>
       <right/>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -214,24 +235,6 @@
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
@@ -369,53 +372,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color theme="0" tint="-0.249977111117893"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="dotted">
-        <color theme="0" tint="-0.249977111117893"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="dotted">
-        <color theme="0" tint="-0.249977111117893"/>
-      </left>
-      <right style="dotted">
-        <color theme="0" tint="-0.249977111117893"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="0" tint="-0.249977111117893"/>
-      </top>
-      <bottom style="thin">
-        <color theme="0" tint="-0.249977111117893"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -432,74 +393,116 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -835,7 +838,250 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12A059DC-D337-4629-8F0C-12C22110466C}">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:I12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="10.90625" style="23"/>
+    <col min="2" max="2" width="7.1796875" style="23" customWidth="1"/>
+    <col min="3" max="3" width="37.81640625" style="23" customWidth="1"/>
+    <col min="4" max="4" width="30.26953125" style="23" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.54296875" style="23" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.90625" style="23"/>
+    <col min="7" max="7" width="42.08984375" style="23" customWidth="1"/>
+    <col min="8" max="8" width="12.81640625" style="24" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="10.90625" style="23"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A1" s="22" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="22"/>
+    </row>
+    <row r="3" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B4" s="25" t="s">
+        <v>32</v>
+      </c>
+      <c r="C4" s="26" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="26" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="G4" s="27" t="s">
+        <v>5</v>
+      </c>
+      <c r="H4" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="I4" s="28" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="B5" s="29">
+        <v>1</v>
+      </c>
+      <c r="C5" s="30" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" s="31" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" s="31" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="H5" s="30" t="s">
+        <v>17</v>
+      </c>
+      <c r="I5" s="32" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="B6" s="29">
+        <v>2</v>
+      </c>
+      <c r="C6" s="30" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" s="31" t="s">
+        <v>8</v>
+      </c>
+      <c r="G6" s="30" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" s="30" t="s">
+        <v>17</v>
+      </c>
+      <c r="I6" s="32" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="58" x14ac:dyDescent="0.35">
+      <c r="B7" s="33">
+        <v>3</v>
+      </c>
+      <c r="C7" s="34" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="34" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="35" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" s="35" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="34" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" s="34" t="s">
+        <v>18</v>
+      </c>
+      <c r="I7" s="36" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="B8" s="33">
+        <v>4</v>
+      </c>
+      <c r="C8" s="34" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" s="34" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="35"/>
+      <c r="G8" s="34" t="s">
+        <v>31</v>
+      </c>
+      <c r="H8" s="34" t="s">
+        <v>37</v>
+      </c>
+      <c r="I8" s="36" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="B9" s="33">
+        <v>5</v>
+      </c>
+      <c r="C9" s="34" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="34" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="35" t="s">
+        <v>21</v>
+      </c>
+      <c r="G9" s="34" t="s">
+        <v>22</v>
+      </c>
+      <c r="H9" s="34" t="s">
+        <v>30</v>
+      </c>
+      <c r="I9" s="36" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="B10" s="29">
+        <v>6</v>
+      </c>
+      <c r="C10" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="E10" s="31" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="31" t="s">
+        <v>21</v>
+      </c>
+      <c r="G10" s="30" t="s">
+        <v>24</v>
+      </c>
+      <c r="H10" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="I10" s="32" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B11" s="37">
+        <v>7</v>
+      </c>
+      <c r="C11" s="38" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="38" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="38" t="s">
+        <v>28</v>
+      </c>
+      <c r="G11" s="39" t="s">
+        <v>29</v>
+      </c>
+      <c r="H11" s="39" t="s">
+        <v>30</v>
+      </c>
+      <c r="I11" s="40" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B12" s="41"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="41"/>
+      <c r="G12" s="41"/>
+      <c r="H12" s="42"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7CC63B2-8A06-4585-8D65-E8CED54E6601}">
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.90625" style="2"/>
@@ -844,199 +1090,225 @@
     <col min="4" max="4" width="27.6328125" style="2" customWidth="1"/>
     <col min="5" max="5" width="11.54296875" style="2" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.90625" style="2"/>
-    <col min="7" max="7" width="36" style="2" customWidth="1"/>
-    <col min="8" max="8" width="14.08984375" style="3" customWidth="1"/>
+    <col min="7" max="7" width="42.08984375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="12.81640625" style="3" bestFit="1" customWidth="1"/>
     <col min="9" max="16384" width="10.90625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="20"/>
-    </row>
-    <row r="3" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B4" s="28" t="s">
+      <c r="C1" s="1"/>
+    </row>
+    <row r="3" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B4" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="E4" s="14" t="s">
+      <c r="E4" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="G4" s="24" t="s">
+      <c r="G4" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="H4" s="8" t="s">
+      <c r="H4" s="20" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="B5" s="11">
+      <c r="I4" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B5" s="10">
         <v>1</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="18" t="s">
+      <c r="E5" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="F5" s="18" t="s">
+      <c r="F5" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="G5" s="25" t="s">
+      <c r="G5" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="H5" s="9" t="s">
+      <c r="H5" s="14" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="B6" s="11">
+      <c r="I5" s="8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="B6" s="10">
         <v>2</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="15" t="s">
+      <c r="D6" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="18" t="s">
+      <c r="E6" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="F6" s="18" t="s">
+      <c r="F6" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="G6" s="25" t="s">
+      <c r="G6" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="H6" s="14" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B7" s="12">
+      <c r="I6" s="8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="B7" s="11">
         <v>3</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="16" t="s">
+      <c r="D7" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="F7" s="19" t="s">
+      <c r="F7" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="26" t="s">
+      <c r="G7" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="H7" s="10" t="s">
+      <c r="H7" s="15" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B8" s="12">
+      <c r="I7" s="9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="B8" s="11">
         <v>4</v>
       </c>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="D8" s="16" t="s">
+      <c r="D8" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="E8" s="19" t="s">
+      <c r="E8" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="F8" s="19"/>
-      <c r="G8" s="26" t="s">
+      <c r="F8" s="18"/>
+      <c r="G8" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="H8" s="10"/>
-    </row>
-    <row r="9" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="B9" s="21">
+      <c r="H8" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="I8" s="9" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="B9" s="11">
         <v>5</v>
       </c>
-      <c r="C9" s="22" t="s">
+      <c r="C9" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="22" t="s">
+      <c r="D9" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="23" t="s">
+      <c r="E9" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="F9" s="23" t="s">
+      <c r="F9" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="G9" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="H9" s="15" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" ht="29" x14ac:dyDescent="0.35">
-      <c r="B10" s="11">
+      <c r="I9" s="9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="B10" s="10">
         <v>6</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="D10" s="15" t="s">
+      <c r="D10" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="E10" s="18" t="s">
+      <c r="E10" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="F10" s="18" t="s">
+      <c r="F10" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="G10" s="25" t="s">
+      <c r="G10" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="H10" s="9" t="s">
+      <c r="H10" s="14" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B11" s="13">
+      <c r="I10" s="8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B11" s="12">
         <v>7</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="C11" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="17" t="s">
+      <c r="D11" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="E11" s="17" t="s">
+      <c r="E11" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="F11" s="17" t="s">
+      <c r="F11" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="G11" s="27" t="s">
+      <c r="G11" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="H11" s="7" t="s">
+      <c r="H11" s="21" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I11" s="6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
       <c r="D12" s="5"/>
@@ -1048,4 +1320,13 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81F8AC51-57EA-4500-9062-024B5FDDBB3D}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>